<commit_message>
Updates, including reorganization and naming convention, updates to TIMS data processing, etc...
</commit_message>
<xml_diff>
--- a/Indicator_Gen/Products/RHNA/config/TOC.xlsx
+++ b/Indicator_Gen/Products/RHNA/config/TOC.xlsx
@@ -1,22 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29029"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jfontes\Documents\Projects\Regional-Monitoring\Indicator_Gen\Products\RHNA\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FA08884E-BB7B-4E9A-A0A6-6FF212D5A9ED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C69F4C3A-93C0-49FB-A04E-1E4E59B12F91}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="57480" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Cycle 7 draft indicators" sheetId="2" r:id="rId1"/>
+    <sheet name="TOC" sheetId="4" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Cycle 7 draft indicators'!$B$1:$D$74</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">TOC!$B$1:$D$86</definedName>
   </definedNames>
   <calcPr calcId="191028"/>
   <extLst>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="390" uniqueCount="247">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="444" uniqueCount="280">
   <si>
     <t>Table Name</t>
   </si>
@@ -410,12 +410,6 @@
     <t>HSG-10</t>
   </si>
   <si>
-    <t>Median Contract Rent</t>
-  </si>
-  <si>
-    <t>U.S. Census Bureau, American Community Survey 5-Year Data releases, starting with 2005-2009 through 2015-2019,  B25058, B25056 (for unincorporated areas). County and regional counts are weighted averages of jurisdiction median using B25003 rental unit counts from the relevant year.</t>
-  </si>
-  <si>
     <t>HSG-11</t>
   </si>
   <si>
@@ -428,9 +422,6 @@
     <t>California Department of Housing and Community Development (HCD), 5th Cycle Annual Progress Report Permit Summary (2020)</t>
   </si>
   <si>
-    <t>HHs by new income bracket</t>
-  </si>
-  <si>
     <t>RISK-01</t>
   </si>
   <si>
@@ -764,15 +755,9 @@
     <t>ELI-04</t>
   </si>
   <si>
-    <t>Forthcoming indicator (i.e. no data yet)</t>
-  </si>
-  <si>
     <t xml:space="preserve">HUD counts are only at CoC geography, so jurisdictions would need to supplement this data with own local estimates. </t>
   </si>
   <si>
-    <t>Not all jurisdictions have data through this source</t>
-  </si>
-  <si>
     <t>Data is at county level. Last cycle HCD accepted at county level, unclear if they will this cycle.SACOG looking into what other farmworker housing data is available</t>
   </si>
   <si>
@@ -780,6 +765,120 @@
   </si>
   <si>
     <t>HOMELS-03</t>
+  </si>
+  <si>
+    <t>POPEMP-26</t>
+  </si>
+  <si>
+    <t>Population Projections</t>
+  </si>
+  <si>
+    <t>Recommended by Users</t>
+  </si>
+  <si>
+    <t>SACOG</t>
+  </si>
+  <si>
+    <t>SACOG Sustainable Communities Strategy regional growth projection series</t>
+  </si>
+  <si>
+    <t>HSG-12</t>
+  </si>
+  <si>
+    <t>FARM-03</t>
+  </si>
+  <si>
+    <t>Farm Employment Through Time</t>
+  </si>
+  <si>
+    <t>FARM-04</t>
+  </si>
+  <si>
+    <t>Farm Worker Share</t>
+  </si>
+  <si>
+    <t>U.S. Census Bureau, American Community Survey 5-Year Data, Table C24030</t>
+  </si>
+  <si>
+    <t>FAMR-05</t>
+  </si>
+  <si>
+    <t>Farm Workers Residing in Jurisdiction</t>
+  </si>
+  <si>
+    <t>FARM-06</t>
+  </si>
+  <si>
+    <t>Farm Worker Income</t>
+  </si>
+  <si>
+    <t>AFFH-04</t>
+  </si>
+  <si>
+    <t>Dissimilarity Index</t>
+  </si>
+  <si>
+    <t>HUD for definition, but may need to use ACS for demographic</t>
+  </si>
+  <si>
+    <t>AFFH-05</t>
+  </si>
+  <si>
+    <t>Languages spoken at home</t>
+  </si>
+  <si>
+    <t>Not Required by HCD, but Recommended by Beta testers</t>
+  </si>
+  <si>
+    <t>Median Age</t>
+  </si>
+  <si>
+    <t>POPEMP-27</t>
+  </si>
+  <si>
+    <t>POPEMP-28</t>
+  </si>
+  <si>
+    <t>Top 10 Employers</t>
+  </si>
+  <si>
+    <t>EDD</t>
+  </si>
+  <si>
+    <t>U.S. Census Bureau, American Community Survey 5-Year Data (2015-2019), Table S0101</t>
+  </si>
+  <si>
+    <t>Employment Development Department (EDD)</t>
+  </si>
+  <si>
+    <t>Zillow, Zillow Home Value Index (ZORI)</t>
+  </si>
+  <si>
+    <t>Zillow Observed Rent Index (ZORI)</t>
+  </si>
+  <si>
+    <t>Median Rent by Unit Size</t>
+  </si>
+  <si>
+    <t>U.S. Census Bureau, American Community Survey 5-Year Data (2015-2019), Table B25031</t>
+  </si>
+  <si>
+    <t>HSG-13</t>
+  </si>
+  <si>
+    <t>Zillow Home Value Index (ZHVI) by Unit Size</t>
+  </si>
+  <si>
+    <t>U.S. Census Bureau, American Community Survey 5-Year Data (2015-2019), Table B16002</t>
+  </si>
+  <si>
+    <t>ELI-05</t>
+  </si>
+  <si>
+    <t>Households by new income bracket</t>
+  </si>
+  <si>
+    <t>Household Income Distribution by Tenure</t>
   </si>
 </sst>
 </file>
@@ -815,21 +914,20 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
       <u/>
       <sz val="11"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF000000"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-    </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -842,8 +940,14 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="11">
     <border>
       <left/>
       <right/>
@@ -866,6 +970,113 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
@@ -874,28 +1085,77 @@
       <protection locked="0"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="40">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1232,14 +1492,14 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{82465F3C-F83F-47D5-BD55-78C7EA8F9BC2}">
-  <dimension ref="A1:G74"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B1E3A83E-B7B5-41BD-9C40-89F5CF1F7C8C}">
+  <dimension ref="A1:G86"/>
   <sheetFormatPr defaultColWidth="9.1796875" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="13.1796875" customWidth="1"/>
     <col min="2" max="2" width="75.1796875" customWidth="1"/>
     <col min="3" max="3" width="47.7265625" customWidth="1"/>
-    <col min="4" max="4" width="21.90625" customWidth="1"/>
+    <col min="4" max="4" width="21.81640625" customWidth="1"/>
     <col min="5" max="5" width="45.7265625" customWidth="1"/>
     <col min="6" max="6" width="22" customWidth="1"/>
     <col min="7" max="7" width="82.1796875" customWidth="1"/>
@@ -1247,9 +1507,9 @@
   <sheetData>
     <row r="1" spans="1:7" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
-        <v>238</v>
-      </c>
-      <c r="B1" s="1" t="s">
+        <v>235</v>
+      </c>
+      <c r="B1" s="29" t="s">
         <v>0</v>
       </c>
       <c r="C1" s="1" t="s">
@@ -1268,20 +1528,20 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:7" ht="14.5" x14ac:dyDescent="0.35">
-      <c r="A2" s="2" t="s">
+    <row r="2" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A2" s="22" t="s">
         <v>6</v>
       </c>
-      <c r="B2" s="3" t="s">
+      <c r="B2" s="30" t="s">
         <v>7</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="C2" s="19" t="s">
         <v>8</v>
       </c>
       <c r="D2" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="E2" s="11" t="s">
+      <c r="E2" s="33" t="s">
         <v>11</v>
       </c>
       <c r="F2" s="2"/>
@@ -1290,1495 +1550,1638 @@
       </c>
     </row>
     <row r="3" spans="1:7" ht="14.5" x14ac:dyDescent="0.35">
-      <c r="A3" s="2" t="s">
+      <c r="A3" s="22" t="s">
         <v>12</v>
       </c>
-      <c r="B3" s="3" t="s">
+      <c r="B3" s="20" t="s">
         <v>13</v>
       </c>
-      <c r="C3" s="2" t="s">
+      <c r="C3" s="19" t="s">
         <v>8</v>
       </c>
       <c r="D3" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="E3" s="11"/>
+      <c r="E3" s="34"/>
       <c r="F3" s="2"/>
       <c r="G3" s="2" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="4" spans="1:7" ht="14.5" x14ac:dyDescent="0.35">
-      <c r="A4" s="2" t="s">
+      <c r="A4" s="17" t="s">
         <v>16</v>
       </c>
-      <c r="B4" s="3" t="s">
+      <c r="B4" s="20" t="s">
         <v>17</v>
       </c>
-      <c r="C4" s="2" t="s">
+      <c r="C4" s="19" t="s">
         <v>8</v>
       </c>
       <c r="D4" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="E4" s="11"/>
+      <c r="E4" s="34"/>
       <c r="F4" s="2"/>
       <c r="G4" s="2" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="5" spans="1:7" ht="14.5" x14ac:dyDescent="0.35">
-      <c r="A5" s="2" t="s">
+      <c r="A5" s="17" t="s">
         <v>20</v>
       </c>
-      <c r="B5" s="3" t="s">
+      <c r="B5" s="20" t="s">
         <v>21</v>
       </c>
-      <c r="C5" s="2" t="s">
+      <c r="C5" s="19" t="s">
         <v>8</v>
       </c>
       <c r="D5" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="E5" s="11"/>
+      <c r="E5" s="34"/>
       <c r="F5" s="2"/>
       <c r="G5" s="2" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="6" spans="1:7" ht="14.5" x14ac:dyDescent="0.35">
-      <c r="A6" s="2" t="s">
+      <c r="A6" s="17" t="s">
         <v>23</v>
       </c>
-      <c r="B6" s="3" t="s">
+      <c r="B6" s="20" t="s">
         <v>24</v>
       </c>
-      <c r="C6" s="2" t="s">
+      <c r="C6" s="19" t="s">
         <v>25</v>
       </c>
       <c r="D6" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="E6" s="11"/>
+      <c r="E6" s="34"/>
       <c r="F6" s="2"/>
       <c r="G6" s="2" t="s">
         <v>26</v>
       </c>
     </row>
     <row r="7" spans="1:7" ht="14.5" x14ac:dyDescent="0.35">
-      <c r="A7" s="2" t="s">
+      <c r="A7" s="17" t="s">
         <v>27</v>
       </c>
-      <c r="B7" s="3" t="s">
+      <c r="B7" s="20" t="s">
         <v>28</v>
       </c>
-      <c r="C7" s="2" t="s">
+      <c r="C7" s="19" t="s">
         <v>8</v>
       </c>
       <c r="D7" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="E7" s="11"/>
+      <c r="E7" s="34"/>
       <c r="F7" s="2"/>
       <c r="G7" s="2" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="8" spans="1:7" ht="14.5" x14ac:dyDescent="0.35">
-      <c r="A8" s="2" t="s">
+      <c r="A8" s="17" t="s">
         <v>30</v>
       </c>
-      <c r="B8" s="3" t="s">
+      <c r="B8" s="20" t="s">
         <v>31</v>
       </c>
-      <c r="C8" s="2" t="s">
+      <c r="C8" s="19" t="s">
         <v>25</v>
       </c>
       <c r="D8" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="E8" s="11"/>
+      <c r="E8" s="34"/>
       <c r="F8" s="2"/>
       <c r="G8" s="2" t="s">
         <v>32</v>
       </c>
     </row>
     <row r="9" spans="1:7" ht="14.5" x14ac:dyDescent="0.35">
-      <c r="A9" s="2" t="s">
+      <c r="A9" s="17" t="s">
         <v>33</v>
       </c>
-      <c r="B9" s="3" t="s">
+      <c r="B9" s="20" t="s">
         <v>34</v>
       </c>
-      <c r="C9" s="2" t="s">
+      <c r="C9" s="19" t="s">
         <v>25</v>
       </c>
       <c r="D9" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="E9" s="11"/>
+      <c r="E9" s="34"/>
       <c r="F9" s="2"/>
       <c r="G9" s="2" t="s">
         <v>35</v>
       </c>
     </row>
     <row r="10" spans="1:7" ht="14.5" x14ac:dyDescent="0.35">
-      <c r="A10" s="2" t="s">
+      <c r="A10" s="17" t="s">
         <v>36</v>
       </c>
-      <c r="B10" s="3" t="s">
+      <c r="B10" s="20" t="s">
         <v>37</v>
       </c>
-      <c r="C10" s="2" t="s">
+      <c r="C10" s="19" t="s">
         <v>25</v>
       </c>
       <c r="D10" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="E10" s="11"/>
+      <c r="E10" s="34"/>
       <c r="F10" s="2"/>
       <c r="G10" s="2" t="s">
         <v>38</v>
       </c>
     </row>
     <row r="11" spans="1:7" ht="14.5" x14ac:dyDescent="0.35">
-      <c r="A11" s="2" t="s">
+      <c r="A11" s="17" t="s">
         <v>39</v>
       </c>
-      <c r="B11" s="3" t="s">
+      <c r="B11" s="20" t="s">
         <v>40</v>
       </c>
-      <c r="C11" s="2" t="s">
+      <c r="C11" s="19" t="s">
         <v>25</v>
       </c>
       <c r="D11" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="E11" s="11"/>
+      <c r="E11" s="34"/>
       <c r="F11" s="2"/>
       <c r="G11" s="2" t="s">
         <v>41</v>
       </c>
     </row>
     <row r="12" spans="1:7" ht="14.5" x14ac:dyDescent="0.35">
-      <c r="A12" s="2" t="s">
+      <c r="A12" s="17" t="s">
         <v>42</v>
       </c>
-      <c r="B12" s="3" t="s">
+      <c r="B12" s="20" t="s">
         <v>43</v>
       </c>
-      <c r="C12" s="2" t="s">
+      <c r="C12" s="19" t="s">
         <v>25</v>
       </c>
       <c r="D12" s="3" t="s">
         <v>44</v>
       </c>
-      <c r="E12" s="11"/>
+      <c r="E12" s="34"/>
       <c r="F12" s="2"/>
       <c r="G12" s="2" t="s">
         <v>45</v>
       </c>
     </row>
     <row r="13" spans="1:7" ht="14.5" x14ac:dyDescent="0.35">
-      <c r="A13" s="2" t="s">
+      <c r="A13" s="17" t="s">
         <v>46</v>
       </c>
-      <c r="B13" s="6" t="s">
+      <c r="B13" s="20" t="s">
         <v>47</v>
       </c>
-      <c r="C13" s="2" t="s">
+      <c r="C13" s="19" t="s">
         <v>25</v>
       </c>
       <c r="D13" s="3" t="s">
         <v>44</v>
       </c>
-      <c r="E13" s="11"/>
+      <c r="E13" s="34"/>
       <c r="F13" s="2"/>
       <c r="G13" s="2" t="s">
         <v>48</v>
       </c>
     </row>
     <row r="14" spans="1:7" ht="14.5" x14ac:dyDescent="0.35">
-      <c r="A14" s="2" t="s">
+      <c r="A14" s="17" t="s">
         <v>49</v>
       </c>
-      <c r="B14" s="3" t="s">
+      <c r="B14" s="20" t="s">
         <v>50</v>
       </c>
-      <c r="C14" s="2" t="s">
+      <c r="C14" s="19" t="s">
         <v>25</v>
       </c>
       <c r="D14" s="3" t="s">
         <v>51</v>
       </c>
-      <c r="E14" s="11"/>
+      <c r="E14" s="34"/>
       <c r="F14" s="2"/>
       <c r="G14" s="2" t="s">
         <v>52</v>
       </c>
     </row>
     <row r="15" spans="1:7" ht="14.5" x14ac:dyDescent="0.35">
-      <c r="A15" s="2" t="s">
+      <c r="A15" s="17" t="s">
         <v>53</v>
       </c>
-      <c r="B15" s="3" t="s">
+      <c r="B15" s="20" t="s">
         <v>54</v>
       </c>
-      <c r="C15" s="2" t="s">
+      <c r="C15" s="19" t="s">
         <v>25</v>
       </c>
       <c r="D15" s="3" t="s">
         <v>44</v>
       </c>
-      <c r="E15" s="11"/>
+      <c r="E15" s="34"/>
       <c r="F15" s="2"/>
       <c r="G15" s="2" t="s">
         <v>55</v>
       </c>
     </row>
     <row r="16" spans="1:7" ht="14.5" x14ac:dyDescent="0.35">
-      <c r="A16" s="2" t="s">
+      <c r="A16" s="17" t="s">
         <v>56</v>
       </c>
-      <c r="B16" s="3" t="s">
+      <c r="B16" s="20" t="s">
         <v>57</v>
       </c>
-      <c r="C16" s="2" t="s">
+      <c r="C16" s="19" t="s">
         <v>58</v>
       </c>
       <c r="D16" s="3" t="s">
         <v>59</v>
       </c>
-      <c r="E16" s="11"/>
+      <c r="E16" s="34"/>
       <c r="F16" s="2"/>
       <c r="G16" s="2" t="s">
         <v>60</v>
       </c>
     </row>
     <row r="17" spans="1:7" ht="14.5" x14ac:dyDescent="0.35">
-      <c r="A17" s="2" t="s">
+      <c r="A17" s="17" t="s">
         <v>61</v>
       </c>
-      <c r="B17" s="3" t="s">
+      <c r="B17" s="20" t="s">
         <v>62</v>
       </c>
-      <c r="C17" s="2" t="s">
+      <c r="C17" s="19" t="s">
         <v>8</v>
       </c>
       <c r="D17" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="E17" s="11"/>
+      <c r="E17" s="34"/>
       <c r="F17" s="2"/>
       <c r="G17" s="2" t="s">
         <v>63</v>
       </c>
     </row>
     <row r="18" spans="1:7" ht="14.5" x14ac:dyDescent="0.35">
-      <c r="A18" s="2" t="s">
+      <c r="A18" s="17" t="s">
         <v>64</v>
       </c>
-      <c r="B18" s="3" t="s">
+      <c r="B18" s="20" t="s">
         <v>65</v>
       </c>
-      <c r="C18" s="2" t="s">
+      <c r="C18" s="19" t="s">
         <v>58</v>
       </c>
       <c r="D18" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="E18" s="11"/>
+      <c r="E18" s="34"/>
       <c r="F18" s="2"/>
       <c r="G18" s="2" t="s">
         <v>66</v>
       </c>
     </row>
     <row r="19" spans="1:7" ht="14.5" x14ac:dyDescent="0.35">
-      <c r="A19" s="2" t="s">
+      <c r="A19" s="17" t="s">
         <v>67</v>
       </c>
-      <c r="B19" s="3" t="s">
+      <c r="B19" s="20" t="s">
         <v>68</v>
       </c>
-      <c r="C19" s="2" t="s">
+      <c r="C19" s="19" t="s">
         <v>25</v>
       </c>
       <c r="D19" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="E19" s="11"/>
+      <c r="E19" s="34"/>
       <c r="F19" s="2"/>
       <c r="G19" s="2" t="s">
         <v>69</v>
       </c>
     </row>
     <row r="20" spans="1:7" ht="14.5" x14ac:dyDescent="0.35">
-      <c r="A20" s="2" t="s">
+      <c r="A20" s="17" t="s">
         <v>70</v>
       </c>
-      <c r="B20" s="3" t="s">
+      <c r="B20" s="20" t="s">
         <v>71</v>
       </c>
-      <c r="C20" s="2" t="s">
+      <c r="C20" s="19" t="s">
         <v>25</v>
       </c>
       <c r="D20" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="E20" s="11"/>
+      <c r="E20" s="34"/>
       <c r="F20" s="2"/>
       <c r="G20" s="2" t="s">
         <v>72</v>
       </c>
     </row>
     <row r="21" spans="1:7" ht="14.5" x14ac:dyDescent="0.35">
-      <c r="A21" s="2" t="s">
+      <c r="A21" s="17" t="s">
         <v>73</v>
       </c>
-      <c r="B21" s="3" t="s">
+      <c r="B21" s="20" t="s">
         <v>74</v>
       </c>
-      <c r="C21" s="2" t="s">
+      <c r="C21" s="19" t="s">
         <v>25</v>
       </c>
       <c r="D21" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="E21" s="11"/>
+      <c r="E21" s="34"/>
       <c r="F21" s="2"/>
       <c r="G21" s="2" t="s">
         <v>75</v>
       </c>
     </row>
     <row r="22" spans="1:7" ht="14.5" x14ac:dyDescent="0.35">
-      <c r="A22" s="2" t="s">
+      <c r="A22" s="17" t="s">
         <v>76</v>
       </c>
-      <c r="B22" s="3" t="s">
+      <c r="B22" s="20" t="s">
         <v>77</v>
       </c>
-      <c r="C22" s="2" t="s">
+      <c r="C22" s="19" t="s">
         <v>58</v>
       </c>
       <c r="D22" s="3" t="s">
         <v>78</v>
       </c>
-      <c r="E22" s="11"/>
+      <c r="E22" s="34"/>
       <c r="F22" s="2"/>
       <c r="G22" s="2" t="s">
         <v>79</v>
       </c>
     </row>
     <row r="23" spans="1:7" ht="14.5" x14ac:dyDescent="0.35">
-      <c r="A23" s="2" t="s">
+      <c r="A23" s="17" t="s">
         <v>80</v>
       </c>
-      <c r="B23" s="3" t="s">
+      <c r="B23" s="20" t="s">
         <v>81</v>
       </c>
-      <c r="C23" s="2" t="s">
+      <c r="C23" s="19" t="s">
         <v>58</v>
       </c>
       <c r="D23" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="E23" s="11"/>
+      <c r="E23" s="34"/>
       <c r="F23" s="2"/>
       <c r="G23" s="2" t="s">
         <v>82</v>
       </c>
     </row>
     <row r="24" spans="1:7" ht="14.5" x14ac:dyDescent="0.35">
-      <c r="A24" s="2" t="s">
+      <c r="A24" s="17" t="s">
         <v>83</v>
       </c>
-      <c r="B24" s="3" t="s">
+      <c r="B24" s="20" t="s">
         <v>84</v>
       </c>
-      <c r="C24" s="2" t="s">
+      <c r="C24" s="19" t="s">
         <v>8</v>
       </c>
       <c r="D24" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="E24" s="11"/>
+      <c r="E24" s="34"/>
       <c r="F24" s="2"/>
       <c r="G24" s="2" t="s">
         <v>85</v>
       </c>
     </row>
     <row r="25" spans="1:7" ht="14.5" x14ac:dyDescent="0.35">
-      <c r="A25" s="2" t="s">
+      <c r="A25" s="17" t="s">
         <v>87</v>
       </c>
-      <c r="B25" s="3" t="s">
+      <c r="B25" s="20" t="s">
         <v>88</v>
       </c>
-      <c r="C25" s="2" t="s">
+      <c r="C25" s="19" t="s">
         <v>25</v>
       </c>
       <c r="D25" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="E25" s="11"/>
+      <c r="E25" s="34"/>
       <c r="F25" s="2"/>
       <c r="G25" s="2" t="s">
         <v>89</v>
       </c>
     </row>
     <row r="26" spans="1:7" ht="24.65" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A26" s="7" t="s">
+      <c r="A26" s="17" t="s">
         <v>90</v>
       </c>
-      <c r="B26" s="8" t="s">
+      <c r="B26" s="20" t="s">
         <v>91</v>
       </c>
-      <c r="C26" s="7" t="s">
+      <c r="C26" s="19" t="s">
         <v>25</v>
       </c>
-      <c r="D26" s="8" t="s">
+      <c r="D26" s="3" t="s">
         <v>92</v>
       </c>
-      <c r="E26" s="11"/>
-      <c r="F26" s="9" t="s">
-        <v>241</v>
-      </c>
+      <c r="E26" s="34"/>
+      <c r="F26" s="7"/>
       <c r="G26" s="2" t="s">
         <v>93</v>
       </c>
     </row>
-    <row r="27" spans="1:7" ht="14.5" x14ac:dyDescent="0.35">
-      <c r="A27" s="2" t="s">
+    <row r="27" spans="1:7" ht="24.65" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A27" s="18" t="s">
+        <v>242</v>
+      </c>
+      <c r="B27" s="21" t="s">
+        <v>243</v>
+      </c>
+      <c r="C27" s="19" t="s">
+        <v>244</v>
+      </c>
+      <c r="D27" s="3" t="s">
+        <v>245</v>
+      </c>
+      <c r="E27" s="34"/>
+      <c r="F27" s="7"/>
+      <c r="G27" s="2" t="s">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" ht="14.5" x14ac:dyDescent="0.35">
+      <c r="A28" s="17" t="s">
+        <v>264</v>
+      </c>
+      <c r="B28" s="21" t="s">
+        <v>263</v>
+      </c>
+      <c r="C28" s="19" t="s">
+        <v>244</v>
+      </c>
+      <c r="D28" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="E28" s="34"/>
+      <c r="F28" s="7"/>
+      <c r="G28" s="2" t="s">
+        <v>268</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7" ht="14.5" x14ac:dyDescent="0.35">
+      <c r="A29" s="23" t="s">
+        <v>265</v>
+      </c>
+      <c r="B29" s="21" t="s">
+        <v>266</v>
+      </c>
+      <c r="C29" s="26" t="s">
+        <v>58</v>
+      </c>
+      <c r="D29" s="11" t="s">
+        <v>267</v>
+      </c>
+      <c r="E29" s="34"/>
+      <c r="F29" s="12"/>
+      <c r="G29" s="10" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7" ht="14.5" x14ac:dyDescent="0.35">
+      <c r="A30" s="17" t="s">
         <v>94</v>
       </c>
-      <c r="B27" s="3" t="s">
+      <c r="B30" s="20" t="s">
         <v>95</v>
       </c>
-      <c r="C27" s="2" t="s">
+      <c r="C30" s="19" t="s">
         <v>8</v>
       </c>
-      <c r="D27" s="3" t="s">
+      <c r="D30" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="E27" s="11" t="s">
+      <c r="E30" s="33" t="s">
         <v>96</v>
       </c>
-      <c r="F27" s="2"/>
-      <c r="G27" s="2" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="28" spans="1:7" ht="14.5" x14ac:dyDescent="0.35">
-      <c r="A28" s="2" t="s">
-        <v>97</v>
-      </c>
-      <c r="B28" s="3" t="s">
-        <v>98</v>
-      </c>
-      <c r="C28" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="D28" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="E28" s="11"/>
-      <c r="F28" s="2"/>
-      <c r="G28" s="2" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="29" spans="1:7" ht="14.5" x14ac:dyDescent="0.35">
-      <c r="A29" s="2" t="s">
-        <v>100</v>
-      </c>
-      <c r="B29" s="3" t="s">
-        <v>101</v>
-      </c>
-      <c r="C29" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="D29" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="E29" s="11"/>
-      <c r="F29" s="2"/>
-      <c r="G29" s="2" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="30" spans="1:7" ht="14.5" x14ac:dyDescent="0.35">
-      <c r="A30" s="2" t="s">
-        <v>103</v>
-      </c>
-      <c r="B30" s="3" t="s">
-        <v>104</v>
-      </c>
-      <c r="C30" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="D30" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="E30" s="11"/>
       <c r="F30" s="2"/>
       <c r="G30" s="2" t="s">
-        <v>105</v>
+        <v>10</v>
       </c>
     </row>
     <row r="31" spans="1:7" ht="14.5" x14ac:dyDescent="0.35">
-      <c r="A31" s="2" t="s">
-        <v>106</v>
-      </c>
-      <c r="B31" s="3" t="s">
-        <v>107</v>
-      </c>
-      <c r="C31" s="2" t="s">
+      <c r="A31" s="17" t="s">
+        <v>97</v>
+      </c>
+      <c r="B31" s="20" t="s">
+        <v>98</v>
+      </c>
+      <c r="C31" s="19" t="s">
         <v>25</v>
       </c>
       <c r="D31" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="E31" s="11"/>
+      <c r="E31" s="34"/>
       <c r="F31" s="2"/>
       <c r="G31" s="2" t="s">
-        <v>108</v>
+        <v>99</v>
       </c>
     </row>
     <row r="32" spans="1:7" ht="14.5" x14ac:dyDescent="0.35">
-      <c r="A32" s="2" t="s">
-        <v>109</v>
-      </c>
-      <c r="B32" s="3" t="s">
-        <v>110</v>
-      </c>
-      <c r="C32" s="2" t="s">
+      <c r="A32" s="17" t="s">
+        <v>100</v>
+      </c>
+      <c r="B32" s="20" t="s">
+        <v>101</v>
+      </c>
+      <c r="C32" s="19" t="s">
         <v>8</v>
       </c>
       <c r="D32" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="E32" s="11"/>
+      <c r="E32" s="34"/>
       <c r="F32" s="2"/>
       <c r="G32" s="2" t="s">
-        <v>111</v>
+        <v>102</v>
       </c>
     </row>
     <row r="33" spans="1:7" ht="14.5" x14ac:dyDescent="0.35">
-      <c r="A33" s="2" t="s">
-        <v>112</v>
-      </c>
-      <c r="B33" s="3" t="s">
-        <v>113</v>
-      </c>
-      <c r="C33" s="2" t="s">
+      <c r="A33" s="17" t="s">
+        <v>103</v>
+      </c>
+      <c r="B33" s="20" t="s">
+        <v>104</v>
+      </c>
+      <c r="C33" s="19" t="s">
         <v>8</v>
       </c>
       <c r="D33" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="E33" s="11"/>
+      <c r="E33" s="34"/>
       <c r="F33" s="2"/>
       <c r="G33" s="2" t="s">
-        <v>114</v>
-      </c>
-    </row>
-    <row r="34" spans="1:7" ht="29" x14ac:dyDescent="0.35">
-      <c r="A34" s="7" t="s">
-        <v>115</v>
-      </c>
-      <c r="B34" s="8" t="s">
-        <v>116</v>
-      </c>
-      <c r="C34" s="7" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="34" spans="1:7" ht="14.5" x14ac:dyDescent="0.35">
+      <c r="A34" s="17" t="s">
+        <v>106</v>
+      </c>
+      <c r="B34" s="20" t="s">
+        <v>107</v>
+      </c>
+      <c r="C34" s="19" t="s">
         <v>25</v>
       </c>
-      <c r="D34" s="8" t="s">
-        <v>117</v>
-      </c>
-      <c r="E34" s="11"/>
-      <c r="F34" s="9" t="s">
-        <v>243</v>
-      </c>
-      <c r="G34" s="1" t="s">
-        <v>118</v>
+      <c r="D34" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="E34" s="34"/>
+      <c r="F34" s="2"/>
+      <c r="G34" s="2" t="s">
+        <v>108</v>
       </c>
     </row>
     <row r="35" spans="1:7" ht="14.5" x14ac:dyDescent="0.35">
-      <c r="A35" s="2" t="s">
-        <v>119</v>
-      </c>
-      <c r="B35" s="3" t="s">
-        <v>120</v>
-      </c>
-      <c r="C35" s="2" t="s">
+      <c r="A35" s="17" t="s">
+        <v>109</v>
+      </c>
+      <c r="B35" s="20" t="s">
+        <v>110</v>
+      </c>
+      <c r="C35" s="19" t="s">
         <v>8</v>
       </c>
       <c r="D35" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="E35" s="11"/>
+      <c r="E35" s="34"/>
       <c r="F35" s="2"/>
       <c r="G35" s="2" t="s">
-        <v>121</v>
+        <v>111</v>
       </c>
     </row>
     <row r="36" spans="1:7" ht="14.5" x14ac:dyDescent="0.35">
-      <c r="A36" s="2" t="s">
-        <v>122</v>
-      </c>
-      <c r="B36" s="3" t="s">
-        <v>123</v>
-      </c>
-      <c r="C36" s="2" t="s">
+      <c r="A36" s="17" t="s">
+        <v>112</v>
+      </c>
+      <c r="B36" s="20" t="s">
+        <v>113</v>
+      </c>
+      <c r="C36" s="19" t="s">
         <v>8</v>
       </c>
       <c r="D36" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="E36" s="11"/>
+      <c r="E36" s="34"/>
       <c r="F36" s="2"/>
       <c r="G36" s="2" t="s">
-        <v>124</v>
+        <v>114</v>
       </c>
     </row>
     <row r="37" spans="1:7" ht="14.5" x14ac:dyDescent="0.35">
-      <c r="A37" s="2" t="s">
-        <v>125</v>
-      </c>
-      <c r="B37" s="3" t="s">
-        <v>126</v>
-      </c>
-      <c r="C37" s="2" t="s">
+      <c r="A37" s="17" t="s">
+        <v>115</v>
+      </c>
+      <c r="B37" s="20" t="s">
+        <v>116</v>
+      </c>
+      <c r="C37" s="19" t="s">
+        <v>25</v>
+      </c>
+      <c r="D37" s="3" t="s">
+        <v>117</v>
+      </c>
+      <c r="E37" s="34"/>
+      <c r="F37" s="7"/>
+      <c r="G37" s="2" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="38" spans="1:7" ht="14.5" x14ac:dyDescent="0.35">
+      <c r="A38" s="17" t="s">
+        <v>119</v>
+      </c>
+      <c r="B38" s="20" t="s">
+        <v>120</v>
+      </c>
+      <c r="C38" s="19" t="s">
         <v>8</v>
       </c>
-      <c r="D37" s="3" t="s">
-        <v>127</v>
-      </c>
-      <c r="E37" s="11"/>
-      <c r="F37" s="2"/>
-      <c r="G37" s="2" t="s">
-        <v>128</v>
-      </c>
-    </row>
-    <row r="38" spans="1:7" ht="29" x14ac:dyDescent="0.35">
-      <c r="A38" s="7" t="s">
-        <v>130</v>
-      </c>
-      <c r="B38" s="8" t="s">
-        <v>131</v>
-      </c>
-      <c r="C38" s="7" t="s">
+      <c r="D38" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="E38" s="34"/>
+      <c r="F38" s="2"/>
+      <c r="G38" s="2" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="39" spans="1:7" ht="14.5" x14ac:dyDescent="0.35">
+      <c r="A39" s="17" t="s">
+        <v>122</v>
+      </c>
+      <c r="B39" s="20" t="s">
+        <v>271</v>
+      </c>
+      <c r="C39" s="19" t="s">
         <v>8</v>
       </c>
-      <c r="D38" s="8" t="s">
-        <v>132</v>
-      </c>
-      <c r="E38" s="4" t="s">
-        <v>134</v>
-      </c>
-      <c r="F38" s="9" t="s">
-        <v>241</v>
-      </c>
-      <c r="G38" s="1" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="39" spans="1:7" ht="14.5" x14ac:dyDescent="0.35">
-      <c r="A39" s="2" t="s">
-        <v>135</v>
-      </c>
-      <c r="B39" s="3" t="s">
-        <v>136</v>
-      </c>
-      <c r="C39" s="2" t="s">
-        <v>8</v>
-      </c>
       <c r="D39" s="3" t="s">
-        <v>78</v>
-      </c>
-      <c r="E39" s="11" t="s">
-        <v>137</v>
-      </c>
+        <v>117</v>
+      </c>
+      <c r="E39" s="34"/>
       <c r="F39" s="2"/>
       <c r="G39" s="2" t="s">
-        <v>79</v>
+        <v>270</v>
       </c>
     </row>
     <row r="40" spans="1:7" ht="14.5" x14ac:dyDescent="0.35">
-      <c r="A40" s="2" t="s">
-        <v>138</v>
-      </c>
-      <c r="B40" s="3" t="s">
-        <v>139</v>
-      </c>
-      <c r="C40" s="2" t="s">
+      <c r="A40" s="17" t="s">
+        <v>123</v>
+      </c>
+      <c r="B40" s="20" t="s">
+        <v>124</v>
+      </c>
+      <c r="C40" s="19" t="s">
         <v>8</v>
       </c>
       <c r="D40" s="3" t="s">
-        <v>78</v>
-      </c>
-      <c r="E40" s="11"/>
+        <v>125</v>
+      </c>
+      <c r="E40" s="34"/>
       <c r="F40" s="2"/>
       <c r="G40" s="2" t="s">
-        <v>79</v>
+        <v>126</v>
       </c>
     </row>
     <row r="41" spans="1:7" ht="14.5" x14ac:dyDescent="0.35">
-      <c r="A41" s="2" t="s">
-        <v>140</v>
-      </c>
-      <c r="B41" s="3" t="s">
-        <v>141</v>
-      </c>
-      <c r="C41" s="2" t="s">
-        <v>25</v>
+      <c r="A41" s="18" t="s">
+        <v>247</v>
+      </c>
+      <c r="B41" s="21" t="s">
+        <v>272</v>
+      </c>
+      <c r="C41" s="19" t="s">
+        <v>262</v>
       </c>
       <c r="D41" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="E41" s="11"/>
+      <c r="E41" s="34"/>
       <c r="F41" s="2"/>
       <c r="G41" s="2" t="s">
-        <v>142</v>
+        <v>273</v>
       </c>
     </row>
     <row r="42" spans="1:7" ht="14.5" x14ac:dyDescent="0.35">
-      <c r="A42" s="2" t="s">
-        <v>143</v>
-      </c>
-      <c r="B42" s="3" t="s">
-        <v>144</v>
-      </c>
-      <c r="C42" s="2" t="s">
-        <v>58</v>
+      <c r="A42" s="18" t="s">
+        <v>274</v>
+      </c>
+      <c r="B42" s="20" t="s">
+        <v>275</v>
+      </c>
+      <c r="C42" s="19" t="s">
+        <v>262</v>
       </c>
       <c r="D42" s="3" t="s">
-        <v>78</v>
-      </c>
-      <c r="E42" s="11"/>
+        <v>117</v>
+      </c>
+      <c r="E42" s="35"/>
       <c r="F42" s="2"/>
       <c r="G42" s="2" t="s">
-        <v>79</v>
+        <v>118</v>
       </c>
     </row>
     <row r="43" spans="1:7" ht="14.5" x14ac:dyDescent="0.35">
-      <c r="A43" s="2" t="s">
-        <v>145</v>
-      </c>
-      <c r="B43" s="3" t="s">
-        <v>146</v>
-      </c>
-      <c r="C43" s="2" t="s">
+      <c r="A43" s="24" t="s">
+        <v>127</v>
+      </c>
+      <c r="B43" s="20" t="s">
+        <v>128</v>
+      </c>
+      <c r="C43" s="27" t="s">
         <v>8</v>
       </c>
-      <c r="D43" s="3" t="s">
+      <c r="D43" s="14" t="s">
+        <v>129</v>
+      </c>
+      <c r="E43" s="15" t="s">
+        <v>131</v>
+      </c>
+      <c r="F43" s="16"/>
+      <c r="G43" s="13" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="44" spans="1:7" ht="14.5" x14ac:dyDescent="0.35">
+      <c r="A44" s="17" t="s">
+        <v>132</v>
+      </c>
+      <c r="B44" s="20" t="s">
+        <v>133</v>
+      </c>
+      <c r="C44" s="19" t="s">
+        <v>8</v>
+      </c>
+      <c r="D44" s="3" t="s">
         <v>78</v>
       </c>
-      <c r="E43" s="11"/>
-      <c r="F43" s="2"/>
-      <c r="G43" s="2" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="44" spans="1:7" ht="14.5" x14ac:dyDescent="0.35">
-      <c r="A44" s="2" t="s">
-        <v>147</v>
-      </c>
-      <c r="B44" s="3" t="s">
-        <v>148</v>
-      </c>
-      <c r="C44" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="D44" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="E44" s="11"/>
+      <c r="E44" s="39" t="s">
+        <v>134</v>
+      </c>
       <c r="F44" s="2"/>
       <c r="G44" s="2" t="s">
-        <v>149</v>
+        <v>79</v>
       </c>
     </row>
     <row r="45" spans="1:7" ht="14.5" x14ac:dyDescent="0.35">
-      <c r="A45" s="2" t="s">
-        <v>150</v>
-      </c>
-      <c r="B45" s="3" t="s">
-        <v>151</v>
-      </c>
-      <c r="C45" s="2" t="s">
+      <c r="A45" s="17" t="s">
+        <v>135</v>
+      </c>
+      <c r="B45" s="20" t="s">
+        <v>136</v>
+      </c>
+      <c r="C45" s="19" t="s">
         <v>8</v>
       </c>
       <c r="D45" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="E45" s="11"/>
+        <v>78</v>
+      </c>
+      <c r="E45" s="39"/>
       <c r="F45" s="2"/>
       <c r="G45" s="2" t="s">
-        <v>149</v>
+        <v>79</v>
       </c>
     </row>
     <row r="46" spans="1:7" ht="14.5" x14ac:dyDescent="0.35">
-      <c r="A46" s="2" t="s">
-        <v>152</v>
-      </c>
-      <c r="B46" s="3" t="s">
-        <v>153</v>
-      </c>
-      <c r="C46" s="2" t="s">
-        <v>58</v>
+      <c r="A46" s="17" t="s">
+        <v>137</v>
+      </c>
+      <c r="B46" s="20" t="s">
+        <v>138</v>
+      </c>
+      <c r="C46" s="19" t="s">
+        <v>25</v>
       </c>
       <c r="D46" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="E46" s="11"/>
+      <c r="E46" s="39"/>
       <c r="F46" s="2"/>
       <c r="G46" s="2" t="s">
-        <v>79</v>
+        <v>139</v>
       </c>
     </row>
     <row r="47" spans="1:7" ht="14.5" x14ac:dyDescent="0.35">
-      <c r="A47" s="2" t="s">
-        <v>154</v>
-      </c>
-      <c r="B47" s="3" t="s">
-        <v>155</v>
-      </c>
-      <c r="C47" s="2" t="s">
+      <c r="A47" s="17" t="s">
+        <v>140</v>
+      </c>
+      <c r="B47" s="20" t="s">
+        <v>141</v>
+      </c>
+      <c r="C47" s="19" t="s">
         <v>58</v>
       </c>
       <c r="D47" s="3" t="s">
         <v>78</v>
       </c>
-      <c r="E47" s="11"/>
+      <c r="E47" s="39"/>
       <c r="F47" s="2"/>
       <c r="G47" s="2" t="s">
         <v>79</v>
       </c>
     </row>
     <row r="48" spans="1:7" ht="14.5" x14ac:dyDescent="0.35">
-      <c r="A48" s="2" t="s">
-        <v>156</v>
-      </c>
-      <c r="B48" s="3" t="s">
-        <v>157</v>
-      </c>
-      <c r="C48" s="2" t="s">
+      <c r="A48" s="17" t="s">
+        <v>142</v>
+      </c>
+      <c r="B48" s="20" t="s">
+        <v>143</v>
+      </c>
+      <c r="C48" s="19" t="s">
         <v>8</v>
       </c>
       <c r="D48" s="3" t="s">
-        <v>158</v>
-      </c>
-      <c r="E48" s="11" t="s">
-        <v>160</v>
-      </c>
+        <v>78</v>
+      </c>
+      <c r="E48" s="39"/>
       <c r="F48" s="2"/>
       <c r="G48" s="2" t="s">
-        <v>159</v>
+        <v>79</v>
       </c>
     </row>
     <row r="49" spans="1:7" ht="14.5" x14ac:dyDescent="0.35">
-      <c r="A49" s="7" t="s">
-        <v>161</v>
-      </c>
-      <c r="B49" s="8" t="s">
-        <v>162</v>
-      </c>
-      <c r="C49" s="7" t="s">
+      <c r="A49" s="17" t="s">
+        <v>144</v>
+      </c>
+      <c r="B49" s="20" t="s">
+        <v>145</v>
+      </c>
+      <c r="C49" s="19" t="s">
         <v>8</v>
       </c>
-      <c r="D49" s="8" t="s">
-        <v>163</v>
-      </c>
-      <c r="E49" s="11"/>
-      <c r="F49" s="10" t="s">
-        <v>244</v>
-      </c>
-      <c r="G49" s="1" t="s">
-        <v>164</v>
+      <c r="D49" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="E49" s="39"/>
+      <c r="F49" s="2"/>
+      <c r="G49" s="2" t="s">
+        <v>146</v>
       </c>
     </row>
     <row r="50" spans="1:7" ht="14.5" x14ac:dyDescent="0.35">
-      <c r="A50" s="2" t="s">
-        <v>165</v>
-      </c>
-      <c r="B50" s="3" t="s">
-        <v>166</v>
-      </c>
-      <c r="C50" s="2" t="s">
+      <c r="A50" s="17" t="s">
+        <v>147</v>
+      </c>
+      <c r="B50" s="20" t="s">
+        <v>148</v>
+      </c>
+      <c r="C50" s="19" t="s">
         <v>8</v>
       </c>
       <c r="D50" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="E50" s="11" t="s">
-        <v>86</v>
-      </c>
+      <c r="E50" s="39"/>
       <c r="F50" s="2"/>
       <c r="G50" s="2" t="s">
-        <v>167</v>
+        <v>146</v>
       </c>
     </row>
     <row r="51" spans="1:7" ht="14.5" x14ac:dyDescent="0.35">
-      <c r="A51" s="2" t="s">
-        <v>168</v>
-      </c>
-      <c r="B51" s="3" t="s">
-        <v>169</v>
-      </c>
-      <c r="C51" s="2" t="s">
-        <v>25</v>
+      <c r="A51" s="17" t="s">
+        <v>149</v>
+      </c>
+      <c r="B51" s="20" t="s">
+        <v>150</v>
+      </c>
+      <c r="C51" s="19" t="s">
+        <v>58</v>
       </c>
       <c r="D51" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="E51" s="11"/>
+      <c r="E51" s="39"/>
       <c r="F51" s="2"/>
       <c r="G51" s="2" t="s">
-        <v>170</v>
+        <v>79</v>
       </c>
     </row>
     <row r="52" spans="1:7" ht="14.5" x14ac:dyDescent="0.35">
-      <c r="A52" s="2" t="s">
-        <v>171</v>
-      </c>
-      <c r="B52" s="3" t="s">
-        <v>172</v>
-      </c>
-      <c r="C52" s="2" t="s">
-        <v>8</v>
+      <c r="A52" s="17" t="s">
+        <v>151</v>
+      </c>
+      <c r="B52" s="20" t="s">
+        <v>152</v>
+      </c>
+      <c r="C52" s="19" t="s">
+        <v>58</v>
       </c>
       <c r="D52" s="3" t="s">
         <v>78</v>
       </c>
-      <c r="E52" s="11"/>
+      <c r="E52" s="39"/>
       <c r="F52" s="2"/>
       <c r="G52" s="2" t="s">
         <v>79</v>
       </c>
     </row>
     <row r="53" spans="1:7" ht="14.5" x14ac:dyDescent="0.35">
-      <c r="A53" s="2" t="s">
-        <v>173</v>
-      </c>
-      <c r="B53" s="3" t="s">
-        <v>174</v>
-      </c>
-      <c r="C53" s="2" t="s">
-        <v>25</v>
+      <c r="A53" s="17" t="s">
+        <v>153</v>
+      </c>
+      <c r="B53" s="20" t="s">
+        <v>154</v>
+      </c>
+      <c r="C53" s="19" t="s">
+        <v>8</v>
       </c>
       <c r="D53" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="E53" s="11"/>
+        <v>155</v>
+      </c>
+      <c r="E53" s="33" t="s">
+        <v>157</v>
+      </c>
       <c r="F53" s="2"/>
       <c r="G53" s="2" t="s">
-        <v>175</v>
+        <v>156</v>
       </c>
     </row>
     <row r="54" spans="1:7" ht="14.5" x14ac:dyDescent="0.35">
-      <c r="A54" s="2" t="s">
-        <v>176</v>
-      </c>
-      <c r="B54" s="3" t="s">
-        <v>177</v>
-      </c>
-      <c r="C54" s="2" t="s">
+      <c r="A54" s="25" t="s">
+        <v>158</v>
+      </c>
+      <c r="B54" s="20" t="s">
+        <v>159</v>
+      </c>
+      <c r="C54" s="28" t="s">
         <v>8</v>
       </c>
-      <c r="D54" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="E54" s="11"/>
-      <c r="F54" s="2"/>
-      <c r="G54" s="2" t="s">
-        <v>178</v>
+      <c r="D54" s="5" t="s">
+        <v>160</v>
+      </c>
+      <c r="E54" s="34"/>
+      <c r="F54" s="6" t="s">
+        <v>239</v>
+      </c>
+      <c r="G54" s="1" t="s">
+        <v>161</v>
       </c>
     </row>
     <row r="55" spans="1:7" ht="14.5" x14ac:dyDescent="0.35">
-      <c r="A55" s="2" t="s">
-        <v>179</v>
-      </c>
-      <c r="B55" s="3" t="s">
-        <v>180</v>
-      </c>
-      <c r="C55" s="2" t="s">
-        <v>8</v>
+      <c r="A55" s="18" t="s">
+        <v>248</v>
+      </c>
+      <c r="B55" s="21" t="s">
+        <v>249</v>
+      </c>
+      <c r="C55" s="19" t="s">
+        <v>58</v>
       </c>
       <c r="D55" s="3" t="s">
-        <v>78</v>
-      </c>
-      <c r="E55" s="11" t="s">
-        <v>181</v>
-      </c>
+        <v>44</v>
+      </c>
+      <c r="E55" s="34"/>
       <c r="F55" s="2"/>
       <c r="G55" s="2" t="s">
-        <v>79</v>
+        <v>45</v>
       </c>
     </row>
     <row r="56" spans="1:7" ht="14.5" x14ac:dyDescent="0.35">
-      <c r="A56" s="2" t="s">
-        <v>182</v>
-      </c>
-      <c r="B56" s="3" t="s">
-        <v>183</v>
-      </c>
-      <c r="C56" s="2" t="s">
-        <v>25</v>
+      <c r="A56" s="18" t="s">
+        <v>250</v>
+      </c>
+      <c r="B56" s="21" t="s">
+        <v>251</v>
+      </c>
+      <c r="C56" s="19" t="s">
+        <v>58</v>
       </c>
       <c r="D56" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="E56" s="11"/>
+      <c r="E56" s="34"/>
       <c r="F56" s="2"/>
-      <c r="G56" s="2" t="s">
-        <v>184</v>
+      <c r="G56" t="s">
+        <v>252</v>
       </c>
     </row>
     <row r="57" spans="1:7" ht="14.5" x14ac:dyDescent="0.35">
-      <c r="A57" s="2" t="s">
-        <v>185</v>
-      </c>
-      <c r="B57" s="3" t="s">
-        <v>186</v>
-      </c>
-      <c r="C57" s="2" t="s">
+      <c r="A57" s="18" t="s">
+        <v>253</v>
+      </c>
+      <c r="B57" s="21" t="s">
+        <v>254</v>
+      </c>
+      <c r="C57" s="19" t="s">
         <v>58</v>
       </c>
       <c r="D57" s="3" t="s">
-        <v>78</v>
-      </c>
-      <c r="E57" s="11"/>
+        <v>44</v>
+      </c>
+      <c r="E57" s="34"/>
       <c r="F57" s="2"/>
       <c r="G57" s="2" t="s">
-        <v>79</v>
+        <v>48</v>
       </c>
     </row>
     <row r="58" spans="1:7" ht="14.5" x14ac:dyDescent="0.35">
-      <c r="A58" s="2" t="s">
-        <v>187</v>
-      </c>
-      <c r="B58" s="3" t="s">
-        <v>188</v>
-      </c>
-      <c r="C58" s="2" t="s">
-        <v>25</v>
+      <c r="A58" s="18" t="s">
+        <v>255</v>
+      </c>
+      <c r="B58" s="21" t="s">
+        <v>256</v>
+      </c>
+      <c r="C58" s="19" t="s">
+        <v>58</v>
       </c>
       <c r="D58" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="E58" s="11"/>
+      <c r="E58" s="35"/>
       <c r="F58" s="2"/>
-      <c r="G58" s="2" t="s">
-        <v>189</v>
-      </c>
+      <c r="G58" s="1"/>
     </row>
     <row r="59" spans="1:7" ht="14.5" x14ac:dyDescent="0.35">
-      <c r="A59" s="2" t="s">
-        <v>190</v>
-      </c>
-      <c r="B59" s="3" t="s">
-        <v>191</v>
-      </c>
-      <c r="C59" s="2" t="s">
+      <c r="A59" s="17" t="s">
+        <v>162</v>
+      </c>
+      <c r="B59" s="20" t="s">
+        <v>163</v>
+      </c>
+      <c r="C59" s="19" t="s">
         <v>8</v>
       </c>
       <c r="D59" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="E59" s="11" t="s">
-        <v>192</v>
+      <c r="E59" s="39" t="s">
+        <v>86</v>
       </c>
       <c r="F59" s="2"/>
       <c r="G59" s="2" t="s">
-        <v>189</v>
+        <v>164</v>
       </c>
     </row>
     <row r="60" spans="1:7" ht="14.5" x14ac:dyDescent="0.35">
-      <c r="A60" s="2" t="s">
-        <v>193</v>
-      </c>
-      <c r="B60" s="3" t="s">
-        <v>194</v>
-      </c>
-      <c r="C60" s="2" t="s">
-        <v>8</v>
+      <c r="A60" s="17" t="s">
+        <v>165</v>
+      </c>
+      <c r="B60" s="20" t="s">
+        <v>166</v>
+      </c>
+      <c r="C60" s="19" t="s">
+        <v>25</v>
       </c>
       <c r="D60" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="E60" s="11"/>
+      <c r="E60" s="39"/>
       <c r="F60" s="2"/>
       <c r="G60" s="2" t="s">
-        <v>195</v>
+        <v>167</v>
       </c>
     </row>
     <row r="61" spans="1:7" ht="14.5" x14ac:dyDescent="0.35">
-      <c r="A61" s="2" t="s">
-        <v>196</v>
-      </c>
-      <c r="B61" s="3" t="s">
-        <v>197</v>
-      </c>
-      <c r="C61" s="2" t="s">
-        <v>25</v>
+      <c r="A61" s="17" t="s">
+        <v>168</v>
+      </c>
+      <c r="B61" s="20" t="s">
+        <v>169</v>
+      </c>
+      <c r="C61" s="19" t="s">
+        <v>8</v>
       </c>
       <c r="D61" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="E61" s="11"/>
+        <v>78</v>
+      </c>
+      <c r="E61" s="39"/>
       <c r="F61" s="2"/>
       <c r="G61" s="2" t="s">
-        <v>198</v>
-      </c>
-    </row>
-    <row r="62" spans="1:7" ht="29" x14ac:dyDescent="0.35">
-      <c r="A62" s="2" t="s">
-        <v>199</v>
-      </c>
-      <c r="B62" s="3" t="s">
-        <v>200</v>
-      </c>
-      <c r="C62" s="2" t="s">
-        <v>8</v>
+        <v>79</v>
+      </c>
+    </row>
+    <row r="62" spans="1:7" ht="14.5" x14ac:dyDescent="0.35">
+      <c r="A62" s="17" t="s">
+        <v>170</v>
+      </c>
+      <c r="B62" s="20" t="s">
+        <v>171</v>
+      </c>
+      <c r="C62" s="19" t="s">
+        <v>25</v>
       </c>
       <c r="D62" s="3" t="s">
-        <v>201</v>
-      </c>
-      <c r="E62" s="11"/>
+        <v>18</v>
+      </c>
+      <c r="E62" s="39"/>
       <c r="F62" s="2"/>
       <c r="G62" s="2" t="s">
-        <v>202</v>
-      </c>
-    </row>
-    <row r="63" spans="1:7" ht="29" x14ac:dyDescent="0.35">
-      <c r="A63" s="2" t="s">
-        <v>203</v>
-      </c>
-      <c r="B63" s="3" t="s">
-        <v>204</v>
-      </c>
-      <c r="C63" s="2" t="s">
-        <v>58</v>
+        <v>172</v>
+      </c>
+    </row>
+    <row r="63" spans="1:7" ht="14.5" x14ac:dyDescent="0.35">
+      <c r="A63" s="17" t="s">
+        <v>173</v>
+      </c>
+      <c r="B63" s="20" t="s">
+        <v>174</v>
+      </c>
+      <c r="C63" s="19" t="s">
+        <v>8</v>
       </c>
       <c r="D63" s="3" t="s">
-        <v>201</v>
-      </c>
-      <c r="E63" s="11"/>
+        <v>18</v>
+      </c>
+      <c r="E63" s="39"/>
       <c r="F63" s="2"/>
       <c r="G63" s="2" t="s">
-        <v>205</v>
+        <v>175</v>
       </c>
     </row>
     <row r="64" spans="1:7" ht="14.5" x14ac:dyDescent="0.35">
-      <c r="A64" s="7" t="s">
-        <v>206</v>
-      </c>
-      <c r="B64" s="8" t="s">
-        <v>207</v>
-      </c>
-      <c r="C64" s="7" t="s">
+      <c r="A64" s="17" t="s">
+        <v>176</v>
+      </c>
+      <c r="B64" s="20" t="s">
+        <v>177</v>
+      </c>
+      <c r="C64" s="19" t="s">
         <v>8</v>
       </c>
-      <c r="D64" s="8" t="s">
-        <v>208</v>
-      </c>
-      <c r="E64" s="11" t="s">
-        <v>210</v>
-      </c>
-      <c r="F64" s="10" t="s">
-        <v>211</v>
-      </c>
-      <c r="G64" s="1" t="s">
-        <v>209</v>
+      <c r="D64" s="3" t="s">
+        <v>78</v>
+      </c>
+      <c r="E64" s="39" t="s">
+        <v>178</v>
+      </c>
+      <c r="F64" s="2"/>
+      <c r="G64" s="2" t="s">
+        <v>79</v>
       </c>
     </row>
     <row r="65" spans="1:7" ht="14.5" x14ac:dyDescent="0.35">
-      <c r="A65" s="7" t="s">
-        <v>212</v>
-      </c>
-      <c r="B65" s="8" t="s">
-        <v>213</v>
-      </c>
-      <c r="C65" s="7" t="s">
+      <c r="A65" s="17" t="s">
+        <v>179</v>
+      </c>
+      <c r="B65" s="20" t="s">
+        <v>180</v>
+      </c>
+      <c r="C65" s="19" t="s">
+        <v>25</v>
+      </c>
+      <c r="D65" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="E65" s="39"/>
+      <c r="F65" s="2"/>
+      <c r="G65" s="2" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="66" spans="1:7" ht="14.5" x14ac:dyDescent="0.35">
+      <c r="A66" s="17" t="s">
+        <v>182</v>
+      </c>
+      <c r="B66" s="20" t="s">
+        <v>183</v>
+      </c>
+      <c r="C66" s="19" t="s">
         <v>58</v>
       </c>
-      <c r="D65" s="8" t="s">
-        <v>208</v>
-      </c>
-      <c r="E65" s="11"/>
-      <c r="F65" s="10" t="s">
-        <v>242</v>
-      </c>
-      <c r="G65" s="1" t="s">
-        <v>214</v>
-      </c>
-    </row>
-    <row r="66" spans="1:7" ht="14.5" x14ac:dyDescent="0.35">
-      <c r="A66" s="7" t="s">
-        <v>246</v>
-      </c>
-      <c r="B66" s="8" t="s">
-        <v>216</v>
-      </c>
-      <c r="C66" s="7" t="s">
-        <v>58</v>
-      </c>
-      <c r="D66" s="8" t="s">
-        <v>208</v>
-      </c>
-      <c r="E66" s="11"/>
-      <c r="F66" s="10" t="s">
-        <v>245</v>
-      </c>
-      <c r="G66" s="1" t="s">
-        <v>209</v>
-      </c>
-    </row>
-    <row r="67" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A67" s="2" t="s">
-        <v>215</v>
-      </c>
-      <c r="B67" s="3" t="s">
-        <v>217</v>
-      </c>
-      <c r="C67" s="2" t="s">
+      <c r="D66" s="3" t="s">
+        <v>78</v>
+      </c>
+      <c r="E66" s="39"/>
+      <c r="F66" s="2"/>
+      <c r="G66" s="2" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="67" spans="1:7" ht="14.5" x14ac:dyDescent="0.35">
+      <c r="A67" s="17" t="s">
+        <v>184</v>
+      </c>
+      <c r="B67" s="20" t="s">
+        <v>185</v>
+      </c>
+      <c r="C67" s="19" t="s">
         <v>25</v>
       </c>
       <c r="D67" s="3" t="s">
-        <v>158</v>
-      </c>
-      <c r="E67" s="11"/>
+        <v>18</v>
+      </c>
+      <c r="E67" s="39"/>
       <c r="F67" s="2"/>
       <c r="G67" s="2" t="s">
-        <v>159</v>
+        <v>186</v>
       </c>
     </row>
     <row r="68" spans="1:7" ht="14.5" x14ac:dyDescent="0.35">
-      <c r="A68" s="2" t="s">
-        <v>218</v>
-      </c>
-      <c r="B68" s="3" t="s">
-        <v>219</v>
-      </c>
-      <c r="C68" s="2" t="s">
+      <c r="A68" s="17" t="s">
+        <v>187</v>
+      </c>
+      <c r="B68" s="20" t="s">
+        <v>188</v>
+      </c>
+      <c r="C68" s="19" t="s">
         <v>8</v>
       </c>
       <c r="D68" s="3" t="s">
-        <v>78</v>
-      </c>
-      <c r="E68" s="11" t="s">
-        <v>220</v>
+        <v>18</v>
+      </c>
+      <c r="E68" s="39" t="s">
+        <v>189</v>
       </c>
       <c r="F68" s="2"/>
       <c r="G68" s="2" t="s">
-        <v>79</v>
+        <v>186</v>
       </c>
     </row>
     <row r="69" spans="1:7" ht="14.5" x14ac:dyDescent="0.35">
-      <c r="A69" s="2" t="s">
-        <v>221</v>
-      </c>
-      <c r="B69" s="3" t="s">
-        <v>222</v>
-      </c>
-      <c r="C69" s="2" t="s">
-        <v>25</v>
+      <c r="A69" s="17" t="s">
+        <v>190</v>
+      </c>
+      <c r="B69" s="20" t="s">
+        <v>191</v>
+      </c>
+      <c r="C69" s="19" t="s">
+        <v>8</v>
       </c>
       <c r="D69" s="3" t="s">
-        <v>78</v>
-      </c>
-      <c r="E69" s="11"/>
+        <v>18</v>
+      </c>
+      <c r="E69" s="39"/>
       <c r="F69" s="2"/>
       <c r="G69" s="2" t="s">
-        <v>79</v>
+        <v>192</v>
       </c>
     </row>
     <row r="70" spans="1:7" ht="14.5" x14ac:dyDescent="0.35">
-      <c r="A70" s="2" t="s">
-        <v>223</v>
-      </c>
-      <c r="B70" s="3" t="s">
-        <v>224</v>
-      </c>
-      <c r="C70" s="2" t="s">
-        <v>58</v>
+      <c r="A70" s="17" t="s">
+        <v>193</v>
+      </c>
+      <c r="B70" s="20" t="s">
+        <v>194</v>
+      </c>
+      <c r="C70" s="19" t="s">
+        <v>25</v>
       </c>
       <c r="D70" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="E70" s="11"/>
+      <c r="E70" s="39"/>
       <c r="F70" s="2"/>
       <c r="G70" s="2" t="s">
-        <v>225</v>
-      </c>
-    </row>
-    <row r="71" spans="1:7" ht="14.5" x14ac:dyDescent="0.35">
-      <c r="A71" s="2" t="s">
-        <v>240</v>
-      </c>
-      <c r="B71" s="3" t="s">
-        <v>129</v>
-      </c>
-      <c r="C71" s="2" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="71" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+      <c r="A71" s="17" t="s">
+        <v>196</v>
+      </c>
+      <c r="B71" s="20" t="s">
+        <v>197</v>
+      </c>
+      <c r="C71" s="19" t="s">
         <v>8</v>
       </c>
       <c r="D71" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="E71" s="11"/>
+        <v>198</v>
+      </c>
+      <c r="E71" s="39"/>
       <c r="F71" s="2"/>
-      <c r="G71" s="5" t="s">
-        <v>239</v>
-      </c>
-    </row>
-    <row r="72" spans="1:7" ht="14.5" x14ac:dyDescent="0.35">
-      <c r="A72" s="2" t="s">
-        <v>226</v>
-      </c>
-      <c r="B72" s="3" t="s">
-        <v>227</v>
-      </c>
-      <c r="C72" s="2" t="s">
-        <v>25</v>
+      <c r="G71" s="2" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="72" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+      <c r="A72" s="17" t="s">
+        <v>200</v>
+      </c>
+      <c r="B72" s="20" t="s">
+        <v>201</v>
+      </c>
+      <c r="C72" s="19" t="s">
+        <v>58</v>
       </c>
       <c r="D72" s="3" t="s">
-        <v>228</v>
-      </c>
-      <c r="E72" s="12" t="s">
-        <v>230</v>
-      </c>
+        <v>198</v>
+      </c>
+      <c r="E72" s="39"/>
       <c r="F72" s="2"/>
       <c r="G72" s="2" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="73" spans="1:7" ht="14.5" x14ac:dyDescent="0.35">
+      <c r="A73" s="25" t="s">
+        <v>203</v>
+      </c>
+      <c r="B73" s="20" t="s">
+        <v>204</v>
+      </c>
+      <c r="C73" s="28" t="s">
+        <v>8</v>
+      </c>
+      <c r="D73" s="5" t="s">
+        <v>205</v>
+      </c>
+      <c r="E73" s="39" t="s">
+        <v>207</v>
+      </c>
+      <c r="F73" s="6" t="s">
+        <v>208</v>
+      </c>
+      <c r="G73" s="1" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="74" spans="1:7" ht="14.5" x14ac:dyDescent="0.35">
+      <c r="A74" s="25" t="s">
+        <v>209</v>
+      </c>
+      <c r="B74" s="20" t="s">
+        <v>210</v>
+      </c>
+      <c r="C74" s="28" t="s">
+        <v>58</v>
+      </c>
+      <c r="D74" s="5" t="s">
+        <v>205</v>
+      </c>
+      <c r="E74" s="39"/>
+      <c r="F74" s="6" t="s">
+        <v>238</v>
+      </c>
+      <c r="G74" s="1" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="75" spans="1:7" ht="14.5" x14ac:dyDescent="0.35">
+      <c r="A75" s="25" t="s">
+        <v>241</v>
+      </c>
+      <c r="B75" s="20" t="s">
+        <v>213</v>
+      </c>
+      <c r="C75" s="28" t="s">
+        <v>58</v>
+      </c>
+      <c r="D75" s="5" t="s">
+        <v>205</v>
+      </c>
+      <c r="E75" s="39"/>
+      <c r="F75" s="6" t="s">
+        <v>240</v>
+      </c>
+      <c r="G75" s="1" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="76" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A76" s="17" t="s">
+        <v>212</v>
+      </c>
+      <c r="B76" s="20" t="s">
+        <v>214</v>
+      </c>
+      <c r="C76" s="19" t="s">
+        <v>25</v>
+      </c>
+      <c r="D76" s="3" t="s">
+        <v>155</v>
+      </c>
+      <c r="E76" s="39"/>
+      <c r="F76" s="2"/>
+      <c r="G76" s="2" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="77" spans="1:7" ht="14.5" x14ac:dyDescent="0.35">
+      <c r="A77" s="17" t="s">
+        <v>215</v>
+      </c>
+      <c r="B77" s="20" t="s">
+        <v>216</v>
+      </c>
+      <c r="C77" s="19" t="s">
+        <v>8</v>
+      </c>
+      <c r="D77" s="3" t="s">
+        <v>78</v>
+      </c>
+      <c r="E77" s="33" t="s">
+        <v>217</v>
+      </c>
+      <c r="F77" s="2"/>
+      <c r="G77" s="2" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="78" spans="1:7" ht="14.5" x14ac:dyDescent="0.35">
+      <c r="A78" s="17" t="s">
+        <v>218</v>
+      </c>
+      <c r="B78" s="20" t="s">
+        <v>219</v>
+      </c>
+      <c r="C78" s="19" t="s">
+        <v>25</v>
+      </c>
+      <c r="D78" s="3" t="s">
+        <v>78</v>
+      </c>
+      <c r="E78" s="34"/>
+      <c r="F78" s="2"/>
+      <c r="G78" s="2" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="79" spans="1:7" ht="14.5" x14ac:dyDescent="0.35">
+      <c r="A79" s="17" t="s">
+        <v>220</v>
+      </c>
+      <c r="B79" s="20" t="s">
+        <v>221</v>
+      </c>
+      <c r="C79" s="19" t="s">
+        <v>58</v>
+      </c>
+      <c r="D79" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="E79" s="34"/>
+      <c r="F79" s="2"/>
+      <c r="G79" s="2" t="s">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="80" spans="1:7" ht="14.5" x14ac:dyDescent="0.35">
+      <c r="A80" s="17" t="s">
+        <v>237</v>
+      </c>
+      <c r="B80" s="21" t="s">
+        <v>278</v>
+      </c>
+      <c r="C80" s="19" t="s">
+        <v>8</v>
+      </c>
+      <c r="D80" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="E80" s="34"/>
+      <c r="F80" s="2"/>
+      <c r="G80" s="4" t="s">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="81" spans="1:7" ht="14.5" x14ac:dyDescent="0.35">
+      <c r="A81" s="17" t="s">
+        <v>277</v>
+      </c>
+      <c r="B81" s="21" t="s">
+        <v>279</v>
+      </c>
+      <c r="C81" s="19" t="s">
+        <v>58</v>
+      </c>
+      <c r="D81" s="3" t="s">
+        <v>78</v>
+      </c>
+      <c r="E81" s="35"/>
+      <c r="F81" s="19"/>
+      <c r="G81" s="2" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="82" spans="1:7" ht="14.5" x14ac:dyDescent="0.35">
+      <c r="A82" s="17" t="s">
+        <v>223</v>
+      </c>
+      <c r="B82" s="20" t="s">
+        <v>224</v>
+      </c>
+      <c r="C82" s="19" t="s">
+        <v>25</v>
+      </c>
+      <c r="D82" s="32" t="s">
+        <v>225</v>
+      </c>
+      <c r="E82" s="36" t="s">
+        <v>227</v>
+      </c>
+      <c r="F82" s="19"/>
+      <c r="G82" s="2" t="s">
+        <v>226</v>
+      </c>
+    </row>
+    <row r="83" spans="1:7" ht="14.5" x14ac:dyDescent="0.35">
+      <c r="A83" s="17" t="s">
+        <v>228</v>
+      </c>
+      <c r="B83" s="20" t="s">
         <v>229</v>
       </c>
-    </row>
-    <row r="73" spans="1:7" ht="14.5" x14ac:dyDescent="0.35">
-      <c r="A73" s="2" t="s">
+      <c r="C83" s="19" t="s">
+        <v>8</v>
+      </c>
+      <c r="D83" s="32" t="s">
+        <v>230</v>
+      </c>
+      <c r="E83" s="37"/>
+      <c r="F83" s="19"/>
+      <c r="G83" s="2" t="s">
         <v>231</v>
       </c>
-      <c r="B73" s="3" t="s">
+    </row>
+    <row r="84" spans="1:7" ht="14.5" x14ac:dyDescent="0.35">
+      <c r="A84" s="17" t="s">
         <v>232</v>
       </c>
-      <c r="C73" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="D73" s="3" t="s">
+      <c r="B84" s="20" t="s">
         <v>233</v>
       </c>
-      <c r="E73" s="12"/>
-      <c r="F73" s="2"/>
-      <c r="G73" s="2" t="s">
+      <c r="C84" s="19" t="s">
+        <v>25</v>
+      </c>
+      <c r="D84" s="32" t="s">
+        <v>18</v>
+      </c>
+      <c r="E84" s="37"/>
+      <c r="F84" s="19"/>
+      <c r="G84" s="2" t="s">
         <v>234</v>
       </c>
     </row>
-    <row r="74" spans="1:7" ht="14.5" x14ac:dyDescent="0.35">
-      <c r="A74" s="2" t="s">
-        <v>235</v>
-      </c>
-      <c r="B74" s="3" t="s">
-        <v>236</v>
-      </c>
-      <c r="C74" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="D74" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="E74" s="12"/>
-      <c r="F74" s="2"/>
-      <c r="G74" s="2" t="s">
-        <v>237</v>
+    <row r="85" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A85" s="8" t="s">
+        <v>257</v>
+      </c>
+      <c r="B85" s="20" t="s">
+        <v>258</v>
+      </c>
+      <c r="D85" t="s">
+        <v>259</v>
+      </c>
+      <c r="E85" s="37"/>
+      <c r="F85" s="9"/>
+      <c r="G85" s="9"/>
+    </row>
+    <row r="86" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A86" s="8" t="s">
+        <v>260</v>
+      </c>
+      <c r="B86" s="31" t="s">
+        <v>261</v>
+      </c>
+      <c r="C86" s="19" t="s">
+        <v>262</v>
+      </c>
+      <c r="D86" s="32" t="s">
+        <v>18</v>
+      </c>
+      <c r="E86" s="38"/>
+      <c r="F86" s="9"/>
+      <c r="G86" s="2" t="s">
+        <v>276</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="B1:D74" xr:uid="{82465F3C-F83F-47D5-BD55-78C7EA8F9BC2}"/>
+  <autoFilter ref="B1:D86" xr:uid="{82465F3C-F83F-47D5-BD55-78C7EA8F9BC2}"/>
   <mergeCells count="10">
+    <mergeCell ref="E2:E29"/>
+    <mergeCell ref="E30:E42"/>
+    <mergeCell ref="E82:E86"/>
+    <mergeCell ref="E68:E72"/>
+    <mergeCell ref="E73:E76"/>
+    <mergeCell ref="E44:E52"/>
+    <mergeCell ref="E53:E58"/>
     <mergeCell ref="E59:E63"/>
     <mergeCell ref="E64:E67"/>
-    <mergeCell ref="E68:E71"/>
-    <mergeCell ref="E72:E74"/>
-    <mergeCell ref="E2:E26"/>
-    <mergeCell ref="E27:E37"/>
-    <mergeCell ref="E39:E47"/>
-    <mergeCell ref="E48:E49"/>
-    <mergeCell ref="E50:E54"/>
-    <mergeCell ref="E55:E58"/>
+    <mergeCell ref="E77:E81"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink ref="B2" location="'POPEMP-01'!A1" display="Population Growth Trends" xr:uid="{56BB85BD-FC5F-484E-8E39-922AC870FFF6}"/>
-    <hyperlink ref="B3" location="'POPEMP-02'!A1" display="Population by Race, 2000-2019" xr:uid="{634D30D4-137C-41D2-9E92-365E97E93A61}"/>
-    <hyperlink ref="B4" location="'POPEMP-03'!A1" display="Population by Race" xr:uid="{1F77B908-46EE-4D5F-9DA6-0489E73DB4A9}"/>
-    <hyperlink ref="B5" location="'POPEMP-04'!A1" display="Population by Age" xr:uid="{53E038AE-187B-4543-A508-3B5106BA0657}"/>
-    <hyperlink ref="B6" location="'POPEMP-05'!A1" display="Location of Population 1 Year Ago" xr:uid="{2301C409-D30B-4BBA-8F6C-376647F59F32}"/>
-    <hyperlink ref="B7" location="'POPEMP-06'!A1" display="Resident Employment by Industry" xr:uid="{2BD7AC86-AFC6-4B19-B5DC-6703FD607CF1}"/>
-    <hyperlink ref="B8" location="'POPEMP-07'!A1" display="Resident Employment by Occupation" xr:uid="{DE88B032-D7B3-48D2-887C-35F59B943F17}"/>
-    <hyperlink ref="B9" location="'POPEMP-08'!A1" display="Workers, by Class of Worker" xr:uid="{BAEB3F27-A03D-43B4-9E58-654F7F649A32}"/>
-    <hyperlink ref="B10" location="'POPEMP-09'!A1" display="Workers, by Class of Worker, by Place of Work" xr:uid="{4569DE3E-31C7-4FE1-9D59-D3E49F9D2317}"/>
-    <hyperlink ref="B11" location="'POPEMP-10'!A1" display="Workers by Earnings, by Jurisdiction as Place of Work and Place of Residence" xr:uid="{BB08BEA8-9FCE-4F8B-BFA5-3402803ED1D2}"/>
-    <hyperlink ref="B12" location="'POPEMP-11'!A1" display="Jobs in a Jurisdiction by Industry" xr:uid="{6EEC4D74-33CD-4DA7-9D44-189ABC0E6A11}"/>
-    <hyperlink ref="B13" location="'POPEMP-12'!A1" display="Job Holders in a Jurisdiction by Industry" xr:uid="{1284CA77-C67C-4E34-A6B9-11FD776E2EFE}"/>
-    <hyperlink ref="B14" location="'POPEMP-13'!A1" display="Jobs-Household Ratio" xr:uid="{120F1C4E-08E1-4231-84CB-1641474A2176}"/>
-    <hyperlink ref="B15" location="'POPEMP-14'!A1" display="Jobs-Worker Ratios, By Wage Group" xr:uid="{0CDBC911-8593-41F1-9742-5C24ADE3EC66}"/>
-    <hyperlink ref="B16" location="'POPEMP-15'!A1" display="Unemployment Rate" xr:uid="{B8420E63-57EF-4B49-888D-616548487D27}"/>
-    <hyperlink ref="B17" location="'POPEMP-16'!A1" display="Housing Tenure" xr:uid="{DCD1D671-4ED6-4890-9C7F-3D01064E68D4}"/>
-    <hyperlink ref="B18" location="'POPEMP-17'!A1" display="Housing Tenure 2000-2019" xr:uid="{F39F3E6A-77AE-4AA6-BE18-1572F09D6AC1}"/>
-    <hyperlink ref="B19" location="'POPEMP-18'!A1" display="Housing Tenure by Age" xr:uid="{51AFE3EF-709D-403D-8D4F-E389416D170B}"/>
-    <hyperlink ref="B20" location="'POPEMP-19'!A1" display="Housing Tenure by Year Moved to Current Residence" xr:uid="{25DE3B4E-1F5E-4A07-A2CE-4D0F25420AD0}"/>
-    <hyperlink ref="B21" location="'POPEMP-20'!A1" display="Housing Tenure by Race of Householder" xr:uid="{D22EF4E4-C17E-4ED9-B025-8A9CCEE4B244}"/>
-    <hyperlink ref="B22" location="'POPEMP-21'!A1" display="Household Income Level by Tenure" xr:uid="{E3EAC64D-6E69-45FD-B3D5-E97DEAB1DEB3}"/>
-    <hyperlink ref="B23" location="'POPEMP-22'!A1" display="Housing Tenure by Housing Type" xr:uid="{4C00270A-D578-4A19-B2CE-FA110402EEA1}"/>
-    <hyperlink ref="B24" location="'POPEMP-23'!A1" display="Household Type" xr:uid="{EF7E1D8A-762E-4B4D-962A-50EDDBA0ED57}"/>
-    <hyperlink ref="B25" location="'POPEMP-24'!A1" display="Households by Presence of Children" xr:uid="{43C0596E-2F11-43F8-B122-491FD484BD02}"/>
-    <hyperlink ref="B26" location="'POPEMP-25'!A1" display="Households by Displacement Risk and Tenure" xr:uid="{208D2E74-3ED8-4957-BE75-69BE01B10D6B}"/>
-    <hyperlink ref="B27" location="'HSG-01'!A1" display="Housing Type Trends" xr:uid="{2ACAC82F-B6D6-46A5-AB88-101D4391274D}"/>
-    <hyperlink ref="B28" location="'HSG-02'!A1" display="Occupancy Status" xr:uid="{86F47095-6CE2-4CFC-9203-6806A6804153}"/>
-    <hyperlink ref="B29" location="'HSG-03'!A1" display="Vacant Units by Type" xr:uid="{4BEDA129-BB24-4033-98FD-2B3F330CCE73}"/>
-    <hyperlink ref="B30" location="'HSG-04'!A1" display="Housing Units by Year Structure Built" xr:uid="{B15EF3BE-A01F-4360-A863-4B9F17F0B729}"/>
-    <hyperlink ref="B31" location="'HSG-05'!A1" display="Housing Units by Number of Bedrooms" xr:uid="{3BA58AD5-8285-4187-87F4-74B24A81CC56}"/>
-    <hyperlink ref="B32" location="'HSG-06'!A1" display="Substandard Housing Issues" xr:uid="{64322E0E-7D48-4F7B-B900-EC09A6253560}"/>
-    <hyperlink ref="B33" location="'HSG-07'!A1" display="Home Values of Owner-Occupied Units" xr:uid="{E8609F9B-BEF1-45B8-92E3-AA3D136759D2}"/>
-    <hyperlink ref="B34" location="'HSG-08'!A1" display="Zillow Home Value Index (ZHVI)" xr:uid="{C64BA40C-B7E6-44D6-91D3-E8C28A66EB60}"/>
-    <hyperlink ref="B35" location="'HSG-09'!A1" display="Contract Rents for Renter-Occupied Units" xr:uid="{A381C62B-02C6-4880-B919-164906986E20}"/>
-    <hyperlink ref="B36" location="'HSG-10'!A1" display="Median Contract Rent" xr:uid="{5492CEBC-8BC0-4C5C-804B-E4BF9F64DB54}"/>
-    <hyperlink ref="B37" location="'HSG-11'!A1" display="Permitted Housing, by Income Level" xr:uid="{F6D5B17E-199D-43F3-BDD2-2144A20EE178}"/>
-    <hyperlink ref="B38" location="'RISK-01'!A1" display="Assisted Units at Risk of Converstion" xr:uid="{072D2046-EB17-4CE8-A166-2D0191A8240B}"/>
-    <hyperlink ref="E38" r:id="rId1" xr:uid="{027A9434-61D6-44A1-933B-501A4B2CA98F}"/>
-    <hyperlink ref="B39" location="'OVER-01'!A1" display="Overcrowding by Tenure and Severity" xr:uid="{FAC2E3BA-D20E-4E28-87AF-96AE8850EE18}"/>
-    <hyperlink ref="B40" location="'OVER-02'!A1" display="Overcrowding Severity" xr:uid="{82C6DCE8-F01F-44EE-B665-482873EE801B}"/>
-    <hyperlink ref="B41" location="'OVER-03'!A1" display="Overcrowding by Race" xr:uid="{A8B65A6C-3199-4E5F-BA57-7A6C1C12D854}"/>
-    <hyperlink ref="B42" location="'OVER-04'!A1" display="Overcrowding by Income Level" xr:uid="{0FEB32B4-0C70-435B-8C1E-77ED0809678E}"/>
-    <hyperlink ref="B43" location="'OVER-05'!A1" display="Cost Burden by Income Level" xr:uid="{17BA1361-927C-451B-AAF5-DAE8F7760F07}"/>
-    <hyperlink ref="B44" location="'OVER-06'!A1" display="Cost Burden by Tenure" xr:uid="{F4369DE8-6A9E-41A7-8182-546E9C6BC2B2}"/>
-    <hyperlink ref="B45" location="'OVER-07'!A1" display="Cost Burden Severity" xr:uid="{43788945-1410-4E77-AE46-DDFF6AB22433}"/>
-    <hyperlink ref="B46" location="'OVER-08'!A1" display="Cost Burden by Race" xr:uid="{78D2429F-43D7-4A63-86DE-C1F2465ECF43}"/>
-    <hyperlink ref="B47" location="'OVER-09'!A1" display="Cost Burden by Household Size" xr:uid="{ED9B9B04-4331-4CAA-8F59-73A2713695E1}"/>
-    <hyperlink ref="B48" location="'FARM-01'!A1" display="Migrant Worker Student Population" xr:uid="{21A2DD30-6F95-413D-A668-0511734C7840}"/>
-    <hyperlink ref="B49" location="'FARM-02'!A1" display="Farm Operations and Farm Labor by County" xr:uid="{A0D2E849-10A5-4F44-ABB5-18EEDB18918D}"/>
-    <hyperlink ref="B50" location="'LGFEM-01'!A1" display="Household Size by Tenure" xr:uid="{D953DD91-EB45-490A-B3D4-172455A32CF8}"/>
-    <hyperlink ref="B51" location="'LGFEM-02'!A1" display="Households by Household Size" xr:uid="{5B4DD28E-D22C-4BB6-ACE2-542BD8CEAFF2}"/>
-    <hyperlink ref="B52" location="'LGFEM-03'!A1" display="Household Size by Household Income Level" xr:uid="{A5B122CC-4C8A-42DB-859D-C5D2782A6EB7}"/>
-    <hyperlink ref="B53" location="'LGFEM-04'!A1" display="Housing Tenure by Household Type" xr:uid="{3F875114-D908-4BB0-A403-09319F627393}"/>
-    <hyperlink ref="B54" location="'LGFEM-05'!A1" display="Female-Headed Households by Poverty Status" xr:uid="{DD7BF602-EAC8-4EB2-B62D-B44E7A87884B}"/>
-    <hyperlink ref="B55" location="'SEN-01'!A1" display="Senior Households by Income and Tenure" xr:uid="{426E2AFB-E161-4A94-8D2C-D11568D55D16}"/>
-    <hyperlink ref="B56" location="'SEN-02'!A1" display="Senior and Youth Population by Race" xr:uid="{527EEC1E-5B19-441A-AE00-69692280705D}"/>
-    <hyperlink ref="B57" location="'SEN-03'!A1" display="Cost-Burdened Senior Households by Income Level" xr:uid="{5399F520-6564-42CC-A1DD-41A2CD8BA8EC}"/>
-    <hyperlink ref="B58" location="'SEN-04'!A1" display="Disability by Type - Seniors (65 and over)" xr:uid="{BFE6BD76-B886-44C3-89B1-4248CA57E330}"/>
-    <hyperlink ref="B59" location="'DISAB-01'!A1" display="Disability by Type" xr:uid="{94DB1798-1938-4DBB-876D-8C5324AC25F9}"/>
-    <hyperlink ref="B60" location="'DISAB-02'!A1" display="Population by Disability Status" xr:uid="{5F5BD10E-64E1-46EC-AD12-C804208EDF26}"/>
-    <hyperlink ref="B61" location="'DISAB-03'!A1" display="Disability Employment Status" xr:uid="{2FAE1A18-1DE0-46F5-B347-E15F5BBE55F8}"/>
-    <hyperlink ref="B62" location="'DISAB-04'!A1" display="Population with Developmental Disabilities by Age" xr:uid="{0CE10883-E6DF-4144-B72E-32C377EBF889}"/>
-    <hyperlink ref="B63" location="'DISAB-05'!A1" display="Population with Developmental Disabilities by Residence" xr:uid="{3B5F6BC1-CF86-4D8F-A287-16A0CBD1A112}"/>
-    <hyperlink ref="B64" location="'HOMELS-01'!A1" display="Homelessness by Household Type and Shelter Status" xr:uid="{D091A3E6-312D-49CE-A5B8-1BE687A5DD75}"/>
-    <hyperlink ref="B65" location="'HOMELS-02'!A1" display="Racial Group Share of General and Homeless Populations" xr:uid="{BC3C95FC-B863-4D9D-9BCA-241932CEDD46}"/>
-    <hyperlink ref="B66" location="'HOMELS-04'!A1" display="Characteristics for the Population Experiencing Homelessness" xr:uid="{1FD0EC81-8DBA-443F-AE7E-84496B17C724}"/>
-    <hyperlink ref="B67" location="'HOMELS-05'!A1" display="Students in Local Public Schools Experiencing Homelessness" xr:uid="{9D5F52B0-1C47-4CF9-8D1E-6F19988302E5}"/>
-    <hyperlink ref="B68" location="'ELI-01'!A1" display="Households by Household Income Level" xr:uid="{0C4ACFF0-9FA1-4AA7-A7BA-F6FC6A9C1729}"/>
-    <hyperlink ref="B69" location="'ELI-02'!A1" display="Household Income Distribution by Race" xr:uid="{DFF2E843-BA48-44CE-A051-038D67465C90}"/>
-    <hyperlink ref="B70" location="'ELI-03'!A1" display="Poverty Status by Race" xr:uid="{EF80F089-AB42-4044-A892-4F2F1F071B29}"/>
-    <hyperlink ref="B72" location="'AFFH-01'!A1" display="Mortgage Applications and Acceptance by Race" xr:uid="{9C04894F-63E1-4071-B9B3-8384FB41928D}"/>
-    <hyperlink ref="B73" location="'AFFH-02'!A1" display="Population Living in High Resource Areas by Race" xr:uid="{CF2799C5-7180-4333-AD1A-64B25624982A}"/>
-    <hyperlink ref="B74" location="'AFFH-03'!A1" display="Population with Limited English Proficiency" xr:uid="{1A099EF8-8D0E-4BBF-BA0F-C7BA10788814}"/>
+    <hyperlink ref="E43" r:id="rId1" xr:uid="{84809C26-0670-482E-8938-BAD3B7B9E151}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId2"/>
@@ -2786,15 +3189,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010052CF2D8E3E532648A9A53BA8B542239D" ma:contentTypeVersion="14" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="a1fb610553ec5defc474bb1f7a0ddc39">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="9ce6b1c7-1e7d-4e54-8192-c843964c72a7" xmlns:ns3="4ae99fea-3ccc-4497-bfcd-e0cb757e7dff" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="2d9d4414e518fb510d6d835712213802" ns2:_="" ns3:_="">
     <xsd:import namespace="9ce6b1c7-1e7d-4e54-8192-c843964c72a7"/>
@@ -3023,7 +3417,7 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <lcf76f155ced4ddcb4097134ff3c332f xmlns="9ce6b1c7-1e7d-4e54-8192-c843964c72a7">
@@ -3034,15 +3428,16 @@
 </p:properties>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{672AC322-139E-4A84-A6F4-CFAB12A1643B}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F8C42BCB-EB27-43F9-B940-23613F0167FD}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -3061,7 +3456,7 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B7BB98AC-E4A5-4360-8360-66970990680B}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
@@ -3076,4 +3471,12 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{672AC322-139E-4A84-A6F4-CFAB12A1643B}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>